<commit_message>
✅ Veri Güncellendi:  - Sat Sep 12 02:26:47 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E412"/>
+  <dimension ref="A1:E413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12366,6 +12366,35 @@
         </is>
       </c>
     </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>NAZ ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>
++90 216 566 80 73</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>
+Merdivenköy, Ortabahar Sk No:22 Apt. 22/A, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>2026-09-12 02:26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Sep 15 02:45:33 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E413"/>
+  <dimension ref="A1:E414"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12395,6 +12395,35 @@
         </is>
       </c>
     </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Eczane Çay</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>
++90 216 384 16 22</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Prof. Dr. Kemal Akgüder Cd. 24/a, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>2026-09-15 02:45</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sun Sep 20 02:41:33 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E414"/>
+  <dimension ref="A1:E415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12424,6 +12424,35 @@
         </is>
       </c>
     </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Kanarya Eczane Optik</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>
++90 216 347 31 58</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, Bağdat Cad. No:145D, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>2026-09-20 02:41</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sun Sep 27 02:51:59 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E415"/>
+  <dimension ref="A1:E416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12453,6 +12453,35 @@
         </is>
       </c>
     </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Ceren Eczanesi</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>
++90 216 350 06 36</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>
+Sahrayı Cedit, Atatürk Cd. No:57/C, 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>2026-09-27 02:51</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Oct  1 03:25:04 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E416"/>
+  <dimension ref="A1:E418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12482,6 +12482,64 @@
         </is>
       </c>
     </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Akif Toprak Eczanesi</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>
++90 530 607 59 00</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Şht. Emin Çölen Sokağı no:16/B, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>2026-10-01 03:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Çigdem Gürsoy Eczanesi</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>
++90 216 410 12 20</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, Şemsettin Günaltay Cd. No:66 D:C, 34742 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>2026-10-01 03:25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sat Oct  3 03:09:54 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E418"/>
+  <dimension ref="A1:E419"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12540,6 +12540,35 @@
         </is>
       </c>
     </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Gece Eczanesi</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>
++90 539 709 57 55</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, Şemsettin Günaltay Cd., 34742 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>2026-10-03 03:09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Oct 13 04:49:23 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E419"/>
+  <dimension ref="A1:E420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12569,6 +12569,35 @@
         </is>
       </c>
     </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Yeditepe eczanesi</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>
++90 216 565 98 57</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>
+Dumlupınar, Hızırbey Cd. no:201a, 34000 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>2026-10-13 04:49</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Oct 15 02:36:30 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E420"/>
+  <dimension ref="A1:E421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12598,6 +12598,35 @@
         </is>
       </c>
     </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Acil nöbetçi eczane kurye 7/24 pharmacy Delivery</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>
++90 538 397 95 98</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>
+Rasimpaşa, yeṣil sok no19, 34716 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>2026-10-15 02:36</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sun Oct 18 02:24:21 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E421"/>
+  <dimension ref="A1:E422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12627,6 +12627,35 @@
         </is>
       </c>
     </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Bilgen Eczanesi - Kadıköy</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>
++90 532 368 47 45</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>
+SAHRAYICEDİT MAH. ATATÜRK CAD, ATATÜRK CADDESİ ÜZERİNDE VESTEL VE DİŞ POLİKLİNİĞİ OLAN 7 NOLU CAN APARTMANINI GEÇTİKTEN HEMEN SONRAKİ SOKAĞIN BAŞI -APARTMANIN YAN TARAFINDAKİ DÜKKANIDIR, Taşlıyol Sk. NO:2 D:1A, 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>2026-10-18 02:24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Oct 22 02:43:23 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E422"/>
+  <dimension ref="A1:E423"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12656,6 +12656,35 @@
         </is>
       </c>
     </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Tutku Eczanesi</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>
++90 533 022 37 52</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>
+Caferağa, Gen. Asım Gündüz Caddesi No:81/A, 34710 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>2026-10-22 02:43</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri Oct 23 02:47:15 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E423"/>
+  <dimension ref="A1:E424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12685,6 +12685,35 @@
         </is>
       </c>
     </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>MERKEZ ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>
++90 216 565 68 13</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>
+Merdivenköy, Hızırbey Cd. No:221/B, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>2026-10-23 02:47</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>